<commit_message>
feat(sis): hoja CSV en el Excel del concentrado municipal, banda del PALOTEO sin huecos y nombre oficial del municipio
- Nueva pestana CSV (CLUES, VARIABLE, VALOR, MES, ANIO, MUNICIPIO) en Arial Nova 11: un renglon por unidad y por clave
  del PALOTEO, con CLUES y VALOR como formulas que apuntan a la celda del PALOTEO.
- PALOTEO: la banda oscura de la fila 1 ya no tiene huecos blancos.
- Titulos con el nombre oficial (QUERETARO con acento, EL MARQUES); fila 1 de SEGUIMIENTO se acomoda al ancho real.
- Pruebas: CSV contra PALOTEO y lo capturado, y caso de El Marques (14 unidades).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Formatos/concentrado_municipal_plantilla.xlsx
+++ b/Formatos/concentrado_municipal_plantilla.xlsx
@@ -6784,10 +6784,10 @@
       <c r="X1" s="5"/>
       <c r="Y1" s="5"/>
       <c r="Z1" s="6"/>
-      <c r="AA1" s="1"/>
-      <c r="AB1" s="1"/>
+      <c r="AA1" s="5"/>
+      <c r="AB1" s="5"/>
       <c r="AC1" s="6"/>
-      <c r="AD1" s="1"/>
+      <c r="AD1" s="5"/>
       <c r="AE1" s="7"/>
       <c r="AF1" s="7"/>
       <c r="AG1" s="7"/>

</xml_diff>